<commit_message>
Đánh số Kết quả mong muốn theo bước tương ứng cho TC Quản lý gói cước
- Áp dụng cho cả 2 file: UC1-UC2 (233 TC) và UC3-UC4 (120 TC)
- Kết quả gắn số bước sinh ra nó theo kiểu file mẫu Quanlykho
- Đánh số bước cho các TC giao diện chuẩn, tách lại bước/kết quả cho 3 TC tranh chấp và phát hành lại

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/testcases/goi-cuoc/web/TCs_GOICUOC_Chitiet_Banhanh_UC3_UC4.xlsx
+++ b/docs/testcases/goi-cuoc/web/TCs_GOICUOC_Chitiet_Banhanh_UC3_UC4.xlsx
@@ -3614,7 +3614,7 @@
       </c>
       <c r="E15" s="685" t="inlineStr">
         <is>
-          <t>Hiển thị màn hình gồm:
+          <t>1. Hiển thị màn hình gồm:
 + Thanh tiêu đề: nút Quay lại, tiêu đề, trạng thái gói, các button thao tác
 + Khối Thông tin cơ bản
 + Khối Thuộc tính
@@ -3651,15 +3651,16 @@
       </c>
       <c r="D16" s="685" t="inlineStr">
         <is>
-          <t>Kiểm tra về bố cục, font chữ, chính tả, màu chữ</t>
+          <t>1. Kiểm tra về bố cục, font chữ, chính tả, màu chữ</t>
         </is>
       </c>
       <c r="E16" s="685" t="inlineStr">
         <is>
-          <t>1. Các label, có độ dài, rộng và khoảng cách bằng nhau, không xô lệch
-2. Các label sử dụng cùng 1 loại font, cỡ chữ, căn lề
-3. Kiểm tra tất cả lỗi về chính tả, cấu trúc câu, ngữ pháp trên màn hình
-4. Form được bố trí hợp lý và dễ sử dụng</t>
+          <t>1. 
+- Các label, có độ dài, rộng và khoảng cách bằng nhau, không xô lệch
+- Các label sử dụng cùng 1 loại font, cỡ chữ, căn lề
+- Kiểm tra tất cả lỗi về chính tả, cấu trúc câu, ngữ pháp trên màn hình
+- Form được bố trí hợp lý và dễ sử dụng</t>
         </is>
       </c>
       <c r="F16" s="683" t="n"/>
@@ -3688,12 +3689,12 @@
       </c>
       <c r="D17" s="685" t="inlineStr">
         <is>
-          <t>Nhấn Tab liên tục</t>
+          <t>1. Nhấn Tab liên tục</t>
         </is>
       </c>
       <c r="E17" s="685" t="inlineStr">
         <is>
-          <t>Con trỏ di chuyển lần lượt qua các button thao tác theo thứ tự: Từ trái qua phải, từ trên xuống dưới; không dừng tại các trường read-only có thể nhập</t>
+          <t>1. Con trỏ di chuyển lần lượt qua các button thao tác theo thứ tự: Từ trái qua phải, từ trên xuống dưới; không dừng tại các trường read-only có thể nhập</t>
         </is>
       </c>
       <c r="F17" s="683" t="n"/>
@@ -3722,12 +3723,12 @@
       </c>
       <c r="D18" s="685" t="inlineStr">
         <is>
-          <t>Nhấn phím Shift-Tab liên tục</t>
+          <t>1. Nhấn phím Shift-Tab liên tục</t>
         </is>
       </c>
       <c r="E18" s="685" t="inlineStr">
         <is>
-          <t>Con trỏ di chuyển ngược lại theo thứ tự: từ dưới lên trên, từ phải qua trái</t>
+          <t>1. Con trỏ di chuyển ngược lại theo thứ tự: từ dưới lên trên, từ phải qua trái</t>
         </is>
       </c>
       <c r="F18" s="683" t="n"/>
@@ -3763,7 +3764,7 @@
       </c>
       <c r="E19" s="685" t="inlineStr">
         <is>
-          <t>Màn hình thu nhỏ, phóng to tương ứng và không bị vỡ giao diện</t>
+          <t>3. Màn hình thu nhỏ, phóng to tương ứng và không bị vỡ giao diện</t>
         </is>
       </c>
       <c r="F19" s="683" t="n"/>
@@ -3820,7 +3821,7 @@
       </c>
       <c r="E21" s="685" t="inlineStr">
         <is>
-          <t>Hiển thị icon mũi tên (←) viền tròn</t>
+          <t>1. Hiển thị icon mũi tên (←) viền tròn</t>
         </is>
       </c>
       <c r="F21" s="683" t="n"/>
@@ -3858,7 +3859,7 @@
       </c>
       <c r="E22" s="685" t="inlineStr">
         <is>
-          <t>Quay lại màn hình Quản lý gói cước</t>
+          <t>1. Quay lại màn hình Quản lý gói cước</t>
         </is>
       </c>
       <c r="F22" s="683" t="n"/>
@@ -3896,7 +3897,7 @@
       </c>
       <c r="E23" s="685" t="inlineStr">
         <is>
-          <t>Quay lại màn hình Quản lý gói cước</t>
+          <t>1. Quay lại màn hình Quản lý gói cước</t>
         </is>
       </c>
       <c r="F23" s="683" t="n"/>
@@ -3938,7 +3939,7 @@
       </c>
       <c r="E24" s="685" t="inlineStr">
         <is>
-          <t>Hiển thị tiêu đề: "Chi tiết gói cước"</t>
+          <t>1. Hiển thị tiêu đề: "Chi tiết gói cước"</t>
         </is>
       </c>
       <c r="F24" s="683" t="n"/>
@@ -3981,7 +3982,7 @@
       </c>
       <c r="E25" s="685" t="inlineStr">
         <is>
-          <t>Hiển thị trạng thái "Nháp"</t>
+          <t>1. Hiển thị trạng thái "Nháp"</t>
         </is>
       </c>
       <c r="F25" s="683" t="n"/>
@@ -4020,7 +4021,7 @@
       </c>
       <c r="E26" s="685" t="inlineStr">
         <is>
-          <t>Hiển thị trạng thái "Đã phát hành"</t>
+          <t>1. Hiển thị trạng thái "Đã phát hành"</t>
         </is>
       </c>
       <c r="F26" s="683" t="n"/>
@@ -4059,7 +4060,7 @@
       </c>
       <c r="E27" s="685" t="inlineStr">
         <is>
-          <t>Hiển thị trạng thái "Đang kinh doanh"</t>
+          <t>1. Hiển thị trạng thái "Đang kinh doanh"</t>
         </is>
       </c>
       <c r="F27" s="683" t="n"/>
@@ -4098,7 +4099,7 @@
       </c>
       <c r="E28" s="685" t="inlineStr">
         <is>
-          <t>Hiển thị trạng thái "Ngừng kinh doanh"</t>
+          <t>1. Hiển thị trạng thái "Ngừng kinh doanh"</t>
         </is>
       </c>
       <c r="F28" s="683" t="n"/>
@@ -4137,7 +4138,7 @@
       </c>
       <c r="E29" s="685" t="inlineStr">
         <is>
-          <t>Trạng thái trên màn chi tiết giống cột Trạng thái tại danh sách</t>
+          <t>2. Trạng thái trên màn chi tiết giống cột Trạng thái tại danh sách</t>
         </is>
       </c>
       <c r="F29" s="683" t="n"/>
@@ -4180,7 +4181,7 @@
       </c>
       <c r="E30" s="685" t="inlineStr">
         <is>
-          <t>Button "Chỉnh sửa" nền đen bo góc, góc phải, enable ở cả 4 trạng thái</t>
+          <t>1. Button "Chỉnh sửa" nền đen bo góc, góc phải, enable ở cả 4 trạng thái</t>
         </is>
       </c>
       <c r="F30" s="683" t="n"/>
@@ -4218,7 +4219,7 @@
       </c>
       <c r="E31" s="685" t="inlineStr">
         <is>
-          <t>Điều hướng sang màn Chỉnh sửa gói cước, hiển thị đúng dữ liệu của gói đang xem</t>
+          <t>1. Điều hướng sang màn Chỉnh sửa gói cước, hiển thị đúng dữ liệu của gói đang xem</t>
         </is>
       </c>
       <c r="F31" s="683" t="n"/>
@@ -4261,7 +4262,7 @@
       </c>
       <c r="E32" s="685" t="inlineStr">
         <is>
-          <t>Button Xoá enable ở tất cả trạng thái</t>
+          <t>1. Button Xoá enable ở tất cả trạng thái</t>
         </is>
       </c>
       <c r="F32" s="683" t="n"/>
@@ -4300,7 +4301,7 @@
       </c>
       <c r="E33" s="685" t="inlineStr">
         <is>
-          <t>Hiển thị popup xác nhận xoá theo UC Xoá gói cước</t>
+          <t>1. Hiển thị popup xác nhận xoá theo UC Xoá gói cước</t>
         </is>
       </c>
       <c r="F33" s="683" t="n"/>
@@ -4340,7 +4341,7 @@
       </c>
       <c r="E34" s="685" t="inlineStr">
         <is>
-          <t>Hệ thống chặn không cho xoá, gói giữ nguyên trạng thái Đang kinh doanh</t>
+          <t>2. Hệ thống chặn không cho xoá, gói giữ nguyên trạng thái Đang kinh doanh</t>
         </is>
       </c>
       <c r="F34" s="683" t="n"/>
@@ -4383,7 +4384,7 @@
       </c>
       <c r="E35" s="685" t="inlineStr">
         <is>
-          <t>Hiển thị button "Phát hành", trạng thái enable</t>
+          <t>1. Hiển thị button "Phát hành", trạng thái enable</t>
         </is>
       </c>
       <c r="F35" s="683" t="n"/>
@@ -4422,7 +4423,7 @@
       </c>
       <c r="E36" s="685" t="inlineStr">
         <is>
-          <t>Không hiển thị button Phát hành</t>
+          <t>1. Không hiển thị button Phát hành</t>
         </is>
       </c>
       <c r="F36" s="683" t="n"/>
@@ -4461,7 +4462,7 @@
       </c>
       <c r="E37" s="685" t="inlineStr">
         <is>
-          <t>Không hiển thị button Phát hành</t>
+          <t>1. Không hiển thị button Phát hành</t>
         </is>
       </c>
       <c r="F37" s="683" t="n"/>
@@ -4500,7 +4501,7 @@
       </c>
       <c r="E38" s="685" t="inlineStr">
         <is>
-          <t>Không hiển thị button Phát hành</t>
+          <t>1. Không hiển thị button Phát hành</t>
         </is>
       </c>
       <c r="F38" s="683" t="n"/>
@@ -4539,7 +4540,7 @@
       </c>
       <c r="E39" s="685" t="inlineStr">
         <is>
-          <t>Hiển thị popup xác nhận phát hành theo UC Ban hành gói cước</t>
+          <t>1. Hiển thị popup xác nhận phát hành theo UC Ban hành gói cước</t>
         </is>
       </c>
       <c r="F39" s="683" t="n"/>
@@ -4578,7 +4579,7 @@
       <c r="L40" s="683" t="n"/>
       <c r="M40" s="683" t="n"/>
     </row>
-    <row r="41" ht="32" customHeight="1" s="668">
+    <row r="41" ht="48" customHeight="1" s="668">
       <c r="A41" s="684">
         <f>$C$4&amp;"-"&amp;TEXT(COUNTA($D$12:D41),"00")</f>
         <v/>
@@ -4600,7 +4601,8 @@
       </c>
       <c r="E41" s="685" t="inlineStr">
         <is>
-          <t>- Tất cả trường nền xám nhạt, disabled
+          <t>1. 
+- Tất cả trường nền xám nhạt, disabled
 - Không cho phép nhập, chọn, thêm hoặc xoá dữ liệu</t>
         </is>
       </c>
@@ -4641,7 +4643,7 @@
       </c>
       <c r="E42" s="685" t="inlineStr">
         <is>
-          <t>Không có bản ghi nào thay đổi (updated_at, updated_by giữ nguyên)</t>
+          <t>3. Không có bản ghi nào thay đổi (updated_at, updated_by giữ nguyên)</t>
         </is>
       </c>
       <c r="F42" s="683" t="n"/>
@@ -4683,7 +4685,7 @@
       </c>
       <c r="E43" s="685" t="inlineStr">
         <is>
-          <t>Label "Mã gói cước *", giá trị text in hoa đúng mã đã tạo</t>
+          <t>1. Label "Mã gói cước *", giá trị text in hoa đúng mã đã tạo</t>
         </is>
       </c>
       <c r="F43" s="683" t="inlineStr">
@@ -4730,7 +4732,7 @@
       </c>
       <c r="E44" s="685" t="inlineStr">
         <is>
-          <t>Hiển thị "tammi"</t>
+          <t>1. Hiển thị "tammi"</t>
         </is>
       </c>
       <c r="F44" s="683" t="inlineStr">
@@ -4773,7 +4775,7 @@
       </c>
       <c r="E45" s="685" t="inlineStr">
         <is>
-          <t>Trường Tag hiển thị rỗng, không lỗi layout</t>
+          <t>1. Trường Tag hiển thị rỗng, không lỗi layout</t>
         </is>
       </c>
       <c r="F45" s="683" t="n"/>
@@ -4815,7 +4817,7 @@
       </c>
       <c r="E46" s="685" t="inlineStr">
         <is>
-          <t>Hiển thị đúng nội dung mô tả đã nhập, giữ định dạng gạch đầu dòng</t>
+          <t>1. Hiển thị đúng nội dung mô tả đã nhập, giữ định dạng gạch đầu dòng</t>
         </is>
       </c>
       <c r="F46" s="683" t="inlineStr">
@@ -4858,7 +4860,7 @@
       </c>
       <c r="E47" s="685" t="inlineStr">
         <is>
-          <t>Hiển thị đủ 500 ký tự (có thanh cuộn nếu vượt khung), không vỡ layout</t>
+          <t>1. Hiển thị đủ 500 ký tự (có thanh cuộn nếu vượt khung), không vỡ layout</t>
         </is>
       </c>
       <c r="F47" s="683" t="inlineStr">
@@ -4904,7 +4906,7 @@
       </c>
       <c r="E48" s="685" t="inlineStr">
         <is>
-          <t>Hiển thị đúng giá trị và đơn vị đã lưu khi tạo</t>
+          <t>1. Hiển thị đúng giá trị và đơn vị đã lưu khi tạo</t>
         </is>
       </c>
       <c r="F48" s="683" t="inlineStr">
@@ -4947,7 +4949,7 @@
       </c>
       <c r="E49" s="685" t="inlineStr">
         <is>
-          <t>Hiển thị đúng: 2 - Tuần, 12 - Tháng, 1 - Năm</t>
+          <t>1. Hiển thị đúng: 2 - Tuần, 12 - Tháng, 1 - Năm</t>
         </is>
       </c>
       <c r="F49" s="683" t="n"/>
@@ -4989,7 +4991,7 @@
       </c>
       <c r="E50" s="685" t="inlineStr">
         <is>
-          <t>Hiển thị số tiền có dấu chấm phân cách hàng nghìn</t>
+          <t>1. Hiển thị số tiền có dấu chấm phân cách hàng nghìn</t>
         </is>
       </c>
       <c r="F50" s="683" t="inlineStr">
@@ -5032,7 +5034,7 @@
       </c>
       <c r="E51" s="685" t="inlineStr">
         <is>
-          <t>Hiển thị đủ "9.999.999.999.999", không vỡ layout</t>
+          <t>1. Hiển thị đủ "9.999.999.999.999", không vỡ layout</t>
         </is>
       </c>
       <c r="F51" s="683" t="n"/>
@@ -5074,7 +5076,7 @@
       </c>
       <c r="E52" s="685" t="inlineStr">
         <is>
-          <t>Hiển thị "VNĐ"</t>
+          <t>1. Hiển thị "VNĐ"</t>
         </is>
       </c>
       <c r="F52" s="683" t="n"/>
@@ -5116,7 +5118,7 @@
       </c>
       <c r="E53" s="685" t="inlineStr">
         <is>
-          <t>Hiển thị họ tên Admin cập nhật gói gần nhất</t>
+          <t>1. Hiển thị họ tên Admin cập nhật gói gần nhất</t>
         </is>
       </c>
       <c r="F53" s="683" t="n"/>
@@ -5158,7 +5160,7 @@
       </c>
       <c r="E54" s="685" t="inlineStr">
         <is>
-          <t>Hiển thị thời gian cập nhật gần nhất, định dạng DD/MM/YYYY HH:mm:ss</t>
+          <t>1. Hiển thị thời gian cập nhật gần nhất, định dạng DD/MM/YYYY HH:mm:ss</t>
         </is>
       </c>
       <c r="F54" s="683" t="n"/>
@@ -5197,7 +5199,7 @@
       </c>
       <c r="E55" s="685" t="inlineStr">
         <is>
-          <t>Người cập nhật = Admin B, Thời gian cập nhật = thời điểm phát hành</t>
+          <t>2. Người cập nhật = Admin B, Thời gian cập nhật = thời điểm phát hành</t>
         </is>
       </c>
       <c r="F55" s="683" t="n"/>
@@ -5259,7 +5261,7 @@
       </c>
       <c r="E57" s="685" t="inlineStr">
         <is>
-          <t>Radio "Gói chính" được chọn, "Gói add-on" không chọn, cả 2 disabled</t>
+          <t>1. Radio "Gói chính" được chọn, "Gói add-on" không chọn, cả 2 disabled</t>
         </is>
       </c>
       <c r="F57" s="683" t="n"/>
@@ -5298,7 +5300,7 @@
       </c>
       <c r="E58" s="685" t="inlineStr">
         <is>
-          <t>Radio "Gói add-on" được chọn, disabled</t>
+          <t>1. Radio "Gói add-on" được chọn, disabled</t>
         </is>
       </c>
       <c r="F58" s="683" t="n"/>
@@ -5341,7 +5343,7 @@
       </c>
       <c r="E59" s="685" t="inlineStr">
         <is>
-          <t>Checkbox "Web OA" được tích, "Miniapp gói cước TAMMI" không tích, disabled</t>
+          <t>1. Checkbox "Web OA" được tích, "Miniapp gói cước TAMMI" không tích, disabled</t>
         </is>
       </c>
       <c r="F59" s="683" t="n"/>
@@ -5380,7 +5382,7 @@
       </c>
       <c r="E60" s="685" t="inlineStr">
         <is>
-          <t>Cả 2 checkbox được tích, disabled</t>
+          <t>1. Cả 2 checkbox được tích, disabled</t>
         </is>
       </c>
       <c r="F60" s="683" t="n"/>
@@ -5400,7 +5402,7 @@
         </is>
       </c>
     </row>
-    <row r="61" ht="48" customHeight="1" s="668">
+    <row r="61" ht="64" customHeight="1" s="668">
       <c r="A61" s="684">
         <f>$C$4&amp;"-"&amp;TEXT(COUNTA($D$12:D61),"00")</f>
         <v/>
@@ -5423,7 +5425,8 @@
       </c>
       <c r="E61" s="685" t="inlineStr">
         <is>
-          <t>- "Tự động" được chọn, disabled
+          <t>1. 
+- "Tự động" được chọn, disabled
 - Hiển thị Thời gian bắt đầu, Thời gian kết thúc
 - Không hiển thị Trạng thái kinh doanh</t>
         </is>
@@ -5445,7 +5448,7 @@
         </is>
       </c>
     </row>
-    <row r="62" ht="48" customHeight="1" s="668">
+    <row r="62" ht="64" customHeight="1" s="668">
       <c r="A62" s="684">
         <f>$C$4&amp;"-"&amp;TEXT(COUNTA($D$12:D62),"00")</f>
         <v/>
@@ -5464,7 +5467,8 @@
       </c>
       <c r="E62" s="685" t="inlineStr">
         <is>
-          <t>- "Thủ công" được chọn, disabled
+          <t>1. 
+- "Thủ công" được chọn, disabled
 - Hiển thị Trạng thái kinh doanh
 - Không hiển thị Thời gian bắt đầu, kết thúc</t>
         </is>
@@ -5509,7 +5513,7 @@
       </c>
       <c r="E63" s="685" t="inlineStr">
         <is>
-          <t>Hiển thị đúng thời gian đã lưu, định dạng DD/MM/YYYY hh:mm:ss</t>
+          <t>1. Hiển thị đúng thời gian đã lưu, định dạng DD/MM/YYYY hh:mm:ss</t>
         </is>
       </c>
       <c r="F63" s="683" t="inlineStr">
@@ -5556,7 +5560,7 @@
       </c>
       <c r="E64" s="685" t="inlineStr">
         <is>
-          <t>Hiển thị đúng giá trị đã lưu: "Đang kinh doanh" / "Ngừng kinh doanh"</t>
+          <t>1. Hiển thị đúng giá trị đã lưu: "Đang kinh doanh" / "Ngừng kinh doanh"</t>
         </is>
       </c>
       <c r="F64" s="683" t="n"/>
@@ -5599,7 +5603,7 @@
       </c>
       <c r="E65" s="685" t="inlineStr">
         <is>
-          <t>Hiển thị "1"</t>
+          <t>1. Hiển thị "1"</t>
         </is>
       </c>
       <c r="F65" s="683" t="inlineStr">
@@ -5642,7 +5646,7 @@
       </c>
       <c r="E66" s="685" t="inlineStr">
         <is>
-          <t>Hiển thị rỗng / "0" theo quy ước không giới hạn</t>
+          <t>1. Hiển thị rỗng / "0" theo quy ước không giới hạn</t>
         </is>
       </c>
       <c r="F66" s="683" t="inlineStr">
@@ -5707,7 +5711,7 @@
       </c>
       <c r="E68" s="685" t="inlineStr">
         <is>
-          <t>Hiển thị tên loại gói cước cha, nền xám nhạt</t>
+          <t>1. Hiển thị tên loại gói cước cha, nền xám nhạt</t>
         </is>
       </c>
       <c r="F68" s="683" t="inlineStr">
@@ -5753,7 +5757,7 @@
       </c>
       <c r="E69" s="685" t="inlineStr">
         <is>
-          <t>Hiển thị các cột: STT, Mã tính năng, Tên tính năng, Nhóm tính năng, Tham số, Mô tả, Đánh dấu hiển thị</t>
+          <t>1. Hiển thị các cột: STT, Mã tính năng, Tên tính năng, Nhóm tính năng, Tham số, Mô tả, Đánh dấu hiển thị</t>
         </is>
       </c>
       <c r="F69" s="683" t="n"/>
@@ -5791,7 +5795,7 @@
       </c>
       <c r="E70" s="685" t="inlineStr">
         <is>
-          <t>Hiển thị đủ tính năng thuộc loại gói, không thừa, không thiếu</t>
+          <t>1. Hiển thị đủ tính năng thuộc loại gói, không thừa, không thiếu</t>
         </is>
       </c>
       <c r="F70" s="683" t="n"/>
@@ -5833,7 +5837,7 @@
       </c>
       <c r="E71" s="685" t="inlineStr">
         <is>
-          <t>Số thứ tự tăng dần 1, 2, 3..., căn giữa</t>
+          <t>1. Số thứ tự tăng dần 1, 2, 3..., căn giữa</t>
         </is>
       </c>
       <c r="F71" s="683" t="n"/>
@@ -5875,7 +5879,7 @@
       </c>
       <c r="E72" s="685" t="inlineStr">
         <is>
-          <t>Hiển thị mã tính năng, căn trái</t>
+          <t>1. Hiển thị mã tính năng, căn trái</t>
         </is>
       </c>
       <c r="F72" s="683" t="inlineStr">
@@ -5921,7 +5925,7 @@
       </c>
       <c r="E73" s="685" t="inlineStr">
         <is>
-          <t>Text màu xanh lam dạng hyperlink, căn trái</t>
+          <t>1. Text màu xanh lam dạng hyperlink, căn trái</t>
         </is>
       </c>
       <c r="F73" s="683" t="inlineStr">
@@ -5963,7 +5967,7 @@
       </c>
       <c r="E74" s="685" t="inlineStr">
         <is>
-          <t>Điều hướng đến màn Chi tiết tính năng tương ứng</t>
+          <t>1. Điều hướng đến màn Chi tiết tính năng tương ứng</t>
         </is>
       </c>
       <c r="F74" s="683" t="n"/>
@@ -6005,7 +6009,7 @@
       </c>
       <c r="E75" s="685" t="inlineStr">
         <is>
-          <t>Hiển thị tên nhóm tính năng</t>
+          <t>1. Hiển thị tên nhóm tính năng</t>
         </is>
       </c>
       <c r="F75" s="683" t="inlineStr">
@@ -6051,7 +6055,7 @@
       </c>
       <c r="E76" s="685" t="inlineStr">
         <is>
-          <t>Mỗi tham số là 1 ô con: Tên tham số + (ĐVT: đơn vị) + giá trị bên dưới, read-only</t>
+          <t>1. Mỗi tham số là 1 ô con: Tên tham số + (ĐVT: đơn vị) + giá trị bên dưới, read-only</t>
         </is>
       </c>
       <c r="F76" s="683" t="inlineStr">
@@ -6093,7 +6097,7 @@
       </c>
       <c r="E77" s="685" t="inlineStr">
         <is>
-          <t>Giá trị hiển thị khớp DB</t>
+          <t>1. Giá trị hiển thị khớp DB</t>
         </is>
       </c>
       <c r="F77" s="683" t="n"/>
@@ -6132,7 +6136,7 @@
       </c>
       <c r="E78" s="685" t="inlineStr">
         <is>
-          <t>Hiển thị giá trị Có/Không đúng dữ liệu đã lưu</t>
+          <t>1. Hiển thị giá trị Có/Không đúng dữ liệu đã lưu</t>
         </is>
       </c>
       <c r="F78" s="683" t="n"/>
@@ -6171,7 +6175,7 @@
       </c>
       <c r="E79" s="685" t="inlineStr">
         <is>
-          <t>Hiển thị đủ các ô tham số, không vỡ layout</t>
+          <t>1. Hiển thị đủ các ô tham số, không vỡ layout</t>
         </is>
       </c>
       <c r="F79" s="683" t="n"/>
@@ -6214,7 +6218,7 @@
       </c>
       <c r="E80" s="685" t="inlineStr">
         <is>
-          <t>Hiển thị đầy đủ, không có "…"</t>
+          <t>1. Hiển thị đầy đủ, không có "…"</t>
         </is>
       </c>
       <c r="F80" s="683" t="n"/>
@@ -6253,7 +6257,7 @@
       </c>
       <c r="E81" s="685" t="inlineStr">
         <is>
-          <t>Hiển thị tối đa 2 hàng, phần còn lại thay bằng "…"</t>
+          <t>1. Hiển thị tối đa 2 hàng, phần còn lại thay bằng "…"</t>
         </is>
       </c>
       <c r="F81" s="683" t="n"/>
@@ -6292,7 +6296,7 @@
       </c>
       <c r="E82" s="685" t="inlineStr">
         <is>
-          <t>Hiển thị tooltip chứa toàn bộ mô tả</t>
+          <t>1. Hiển thị tooltip chứa toàn bộ mô tả</t>
         </is>
       </c>
       <c r="F82" s="683" t="n"/>
@@ -6335,7 +6339,7 @@
       </c>
       <c r="E83" s="685" t="inlineStr">
         <is>
-          <t>Tickbox được tích, dòng tính năng hiển thị bình thường</t>
+          <t>1. Tickbox được tích, dòng tính năng hiển thị bình thường</t>
         </is>
       </c>
       <c r="F83" s="683" t="n"/>
@@ -6374,7 +6378,7 @@
       </c>
       <c r="E84" s="685" t="inlineStr">
         <is>
-          <t>Tickbox không tích, dòng tính năng hiển thị ở trạng thái disable</t>
+          <t>1. Tickbox không tích, dòng tính năng hiển thị ở trạng thái disable</t>
         </is>
       </c>
       <c r="F84" s="683" t="n"/>
@@ -6436,7 +6440,7 @@
       </c>
       <c r="E86" s="685" t="inlineStr">
         <is>
-          <t>Hiển thị toast "Thất bại. Vui lòng kiểm tra lại kết nối." và cho phép thử lại</t>
+          <t>2. Hiển thị toast "Thất bại. Vui lòng kiểm tra lại kết nối." và cho phép thử lại</t>
         </is>
       </c>
       <c r="F86" s="683" t="n"/>
@@ -6479,7 +6483,7 @@
       </c>
       <c r="E87" s="685" t="inlineStr">
         <is>
-          <t>Hiển thị toast "Hệ thống bận. Vui lòng thử lại sau." kèm mã lỗi, cho phép thử lại</t>
+          <t>1. Hiển thị toast "Hệ thống bận. Vui lòng thử lại sau." kèm mã lỗi, cho phép thử lại</t>
         </is>
       </c>
       <c r="F87" s="683" t="n"/>
@@ -6522,7 +6526,7 @@
       </c>
       <c r="E88" s="685" t="inlineStr">
         <is>
-          <t>Không hiển thị dữ liệu gói, báo gói không tồn tại / quay về danh sách</t>
+          <t>1. Không hiển thị dữ liệu gói, báo gói không tồn tại / quay về danh sách</t>
         </is>
       </c>
       <c r="F88" s="683" t="n"/>
@@ -6565,7 +6569,7 @@
       </c>
       <c r="E89" s="685" t="inlineStr">
         <is>
-          <t>Toàn bộ dữ liệu khớp CSDL</t>
+          <t>2. Toàn bộ dữ liệu khớp CSDL</t>
         </is>
       </c>
       <c r="F89" s="683" t="n"/>
@@ -6608,7 +6612,7 @@
       </c>
       <c r="E90" s="685" t="inlineStr">
         <is>
-          <t>Bị chặn truy cập</t>
+          <t>1. Bị chặn truy cập</t>
         </is>
       </c>
       <c r="F90" s="683" t="n"/>
@@ -6712,7 +6716,7 @@
       </c>
       <c r="E94" s="685" t="inlineStr">
         <is>
-          <t>Hiển thị popup:
+          <t>2. Hiển thị popup:
 + Icon cảnh báo (!)
 + Tiêu đề: "Phát hành gói cước?"
 + Icon X góc trên bên phải
@@ -6750,15 +6754,16 @@
       </c>
       <c r="D95" s="685" t="inlineStr">
         <is>
-          <t>Kiểm tra về bố cục, font chữ, chính tả, màu chữ</t>
+          <t>1. Kiểm tra về bố cục, font chữ, chính tả, màu chữ</t>
         </is>
       </c>
       <c r="E95" s="685" t="inlineStr">
         <is>
-          <t>1. Các label, có độ dài, rộng và khoảng cách bằng nhau, không xô lệch
-2. Các label sử dụng cùng 1 loại font, cỡ chữ, căn lề
-3. Kiểm tra tất cả lỗi về chính tả, cấu trúc câu, ngữ pháp trên màn hình
-4. Form được bố trí hợp lý và dễ sử dụng</t>
+          <t>1. 
+- Các label, có độ dài, rộng và khoảng cách bằng nhau, không xô lệch
+- Các label sử dụng cùng 1 loại font, cỡ chữ, căn lề
+- Kiểm tra tất cả lỗi về chính tả, cấu trúc câu, ngữ pháp trên màn hình
+- Form được bố trí hợp lý và dễ sử dụng</t>
         </is>
       </c>
       <c r="F95" s="683" t="n"/>
@@ -6793,7 +6798,7 @@
       </c>
       <c r="E96" s="685" t="inlineStr">
         <is>
-          <t>Không thao tác được màn phía sau; popup không đóng</t>
+          <t>1. Không thao tác được màn phía sau; popup không đóng</t>
         </is>
       </c>
       <c r="F96" s="683" t="n"/>
@@ -6855,7 +6860,7 @@
       </c>
       <c r="E98" s="685" t="inlineStr">
         <is>
-          <t>Hiển thị popup:
+          <t>1. Hiển thị popup:
 + Icon cảnh báo (!)
 + Tiêu đề: "Phát hành gói cước?"
 + Icon X góc trên bên phải
@@ -6900,7 +6905,8 @@
       </c>
       <c r="E99" s="685" t="inlineStr">
         <is>
-          <t>- Đóng popup, hiển thị toast "Phát hành gói cước thành công"
+          <t>2. 
+- Đóng popup, hiển thị toast "Phát hành gói cước thành công"
 - Ở lại màn chi tiết, trạng thái gói = "Đã phát hành"
 - Ẩn button Phát hành</t>
         </is>
@@ -6941,7 +6947,7 @@
       </c>
       <c r="E100" s="685" t="inlineStr">
         <is>
-          <t>Gói chưa hiển thị cho người mua</t>
+          <t>1. Gói chưa hiển thị cho người mua</t>
         </is>
       </c>
       <c r="F100" s="683" t="n"/>
@@ -6981,7 +6987,7 @@
       </c>
       <c r="E101" s="685" t="inlineStr">
         <is>
-          <t>Điều hướng đến màn Chỉnh sửa gói cước; trạng thái gói vẫn là Nháp</t>
+          <t>2. Điều hướng đến màn Chỉnh sửa gói cước; trạng thái gói vẫn là Nháp</t>
         </is>
       </c>
       <c r="F101" s="683" t="n"/>
@@ -7021,7 +7027,7 @@
       </c>
       <c r="E102" s="685" t="inlineStr">
         <is>
-          <t>Popup nội dung TH1.1, gói chuyển "Đã phát hành"</t>
+          <t>2. Popup nội dung TH1.1, gói chuyển "Đã phát hành"</t>
         </is>
       </c>
       <c r="F102" s="683" t="inlineStr">
@@ -7069,7 +7075,8 @@
       </c>
       <c r="E103" s="685" t="inlineStr">
         <is>
-          <t>- Trạng thái gói = "Đang kinh doanh"
+          <t>2. 
+- Trạng thái gói = "Đang kinh doanh"
 - Gói hiển thị trên giao diện mua của các kênh đã cấu hình</t>
         </is>
       </c>
@@ -7110,7 +7117,8 @@
       </c>
       <c r="E104" s="685" t="inlineStr">
         <is>
-          <t>- Trạng thái gói = "Ngừng kinh doanh"
+          <t>2. 
+- Trạng thái gói = "Ngừng kinh doanh"
 - Gói không còn hiển thị để mua mới; thuê bao cũ vẫn giữ quyền lợi</t>
         </is>
       </c>
@@ -7154,7 +7162,7 @@
       </c>
       <c r="E105" s="685" t="inlineStr">
         <is>
-          <t>Hiển thị popup:
+          <t>1. Hiển thị popup:
 + Icon cảnh báo (!)
 + Tiêu đề: "Phát hành gói cước?"
 + Icon X góc trên bên phải
@@ -7199,7 +7207,8 @@
       </c>
       <c r="E106" s="685" t="inlineStr">
         <is>
-          <t>- Đóng popup, toast "Phát hành gói cước thành công"
+          <t>2. 
+- Đóng popup, toast "Phát hành gói cước thành công"
 - Trạng thái gói = "Đang kinh doanh"
 - Ẩn button Phát hành</t>
         </is>
@@ -7281,7 +7290,7 @@
       </c>
       <c r="E108" s="685" t="inlineStr">
         <is>
-          <t>Popup nội dung TH1.2 (hiện tại ≥ bắt đầu), xác nhận thì gói chuyển "Đang kinh doanh"</t>
+          <t>1. Popup nội dung TH1.2 (hiện tại ≥ bắt đầu), xác nhận thì gói chuyển "Đang kinh doanh"</t>
         </is>
       </c>
       <c r="F108" s="683" t="n"/>
@@ -7321,7 +7330,7 @@
       </c>
       <c r="E109" s="685" t="inlineStr">
         <is>
-          <t>Điều hướng đến màn Chỉnh sửa gói cước; trạng thái vẫn Nháp</t>
+          <t>2. Điều hướng đến màn Chỉnh sửa gói cước; trạng thái vẫn Nháp</t>
         </is>
       </c>
       <c r="F109" s="683" t="n"/>
@@ -7364,7 +7373,7 @@
       </c>
       <c r="E110" s="685" t="inlineStr">
         <is>
-          <t>Hiển thị popup:
+          <t>1. Hiển thị popup:
 + Icon cảnh báo (!)
 + Tiêu đề: "Phát hành gói cước?"
 + Icon X góc trên bên phải
@@ -7409,7 +7418,8 @@
       </c>
       <c r="E111" s="685" t="inlineStr">
         <is>
-          <t>- Đóng popup, toast "Phát hành gói cước thành công"
+          <t>2. 
+- Đóng popup, toast "Phát hành gói cước thành công"
 - Trạng thái gói = "Ngừng kinh doanh"
 - Gói không hiển thị trên kênh bán</t>
         </is>
@@ -7451,7 +7461,7 @@
       </c>
       <c r="E112" s="685" t="inlineStr">
         <is>
-          <t>Điều hướng đến màn Chỉnh sửa gói cước; trạng thái vẫn Nháp</t>
+          <t>2. Điều hướng đến màn Chỉnh sửa gói cước; trạng thái vẫn Nháp</t>
         </is>
       </c>
       <c r="F112" s="683" t="n"/>
@@ -7490,7 +7500,7 @@
       </c>
       <c r="E113" s="685" t="inlineStr">
         <is>
-          <t>Popup nội dung TH1.3, xác nhận thì gói chuyển "Ngừng kinh doanh"</t>
+          <t>1. Popup nội dung TH1.3, xác nhận thì gói chuyển "Ngừng kinh doanh"</t>
         </is>
       </c>
       <c r="F113" s="683" t="n"/>
@@ -7529,7 +7539,7 @@
       </c>
       <c r="E114" s="685" t="inlineStr">
         <is>
-          <t>Popup nội dung TH1.2 (chưa đến thời gian kết thúc), xác nhận thì gói chuyển "Đang kinh doanh"</t>
+          <t>1. Popup nội dung TH1.2 (chưa đến thời gian kết thúc), xác nhận thì gói chuyển "Đang kinh doanh"</t>
         </is>
       </c>
       <c r="F114" s="683" t="n"/>
@@ -7574,7 +7584,7 @@
       </c>
       <c r="E115" s="685" t="inlineStr">
         <is>
-          <t>Gói chuyển trạng thái theo thời điểm xác nhận (Đang kinh doanh), không kẹt ở Đã phát hành</t>
+          <t>3. Gói chuyển trạng thái theo thời điểm xác nhận (Đang kinh doanh), không kẹt ở Đã phát hành</t>
         </is>
       </c>
       <c r="F115" s="683" t="n"/>
@@ -7636,7 +7646,7 @@
       </c>
       <c r="E117" s="685" t="inlineStr">
         <is>
-          <t>Hiển thị popup:
+          <t>1. Hiển thị popup:
 + Icon cảnh báo (!)
 + Tiêu đề: "Phát hành gói cước?"
 + Icon X góc trên bên phải
@@ -7681,7 +7691,8 @@
       </c>
       <c r="E118" s="685" t="inlineStr">
         <is>
-          <t>- Đóng popup, toast "Phát hành gói cước thành công"
+          <t>2. 
+- Đóng popup, toast "Phát hành gói cước thành công"
 - Trạng thái gói = "Đang kinh doanh"
 - Gói hiển thị ngay trên kênh bán đã cấu hình</t>
         </is>
@@ -7723,7 +7734,7 @@
       </c>
       <c r="E119" s="685" t="inlineStr">
         <is>
-          <t>Điều hướng đến màn Chỉnh sửa gói cước; trạng thái vẫn Nháp</t>
+          <t>2. Điều hướng đến màn Chỉnh sửa gói cước; trạng thái vẫn Nháp</t>
         </is>
       </c>
       <c r="F119" s="683" t="n"/>
@@ -7766,7 +7777,7 @@
       </c>
       <c r="E120" s="685" t="inlineStr">
         <is>
-          <t>Hiển thị popup:
+          <t>1. Hiển thị popup:
 + Icon cảnh báo (!)
 + Tiêu đề: "Phát hành gói cước?"
 + Icon X góc trên bên phải
@@ -7811,7 +7822,8 @@
       </c>
       <c r="E121" s="685" t="inlineStr">
         <is>
-          <t>- Đóng popup, toast "Phát hành gói cước thành công"
+          <t>2. 
+- Đóng popup, toast "Phát hành gói cước thành công"
 - Trạng thái gói = "Ngừng kinh doanh"
 - Gói không hiển thị trên kênh bán</t>
         </is>
@@ -7853,7 +7865,7 @@
       </c>
       <c r="E122" s="685" t="inlineStr">
         <is>
-          <t>Điều hướng đến màn Chỉnh sửa gói cước; trạng thái vẫn Nháp</t>
+          <t>2. Điều hướng đến màn Chỉnh sửa gói cước; trạng thái vẫn Nháp</t>
         </is>
       </c>
       <c r="F122" s="683" t="n"/>
@@ -7897,7 +7909,7 @@
       </c>
       <c r="E123" s="685" t="inlineStr">
         <is>
-          <t>Chỉ căn cứ Trạng thái kinh doanh: gói chuyển "Đang kinh doanh", không hiển thị popup theo thời gian</t>
+          <t>2. Chỉ căn cứ Trạng thái kinh doanh: gói chuyển "Đang kinh doanh", không hiển thị popup theo thời gian</t>
         </is>
       </c>
       <c r="F123" s="683" t="n"/>
@@ -7959,7 +7971,8 @@
       </c>
       <c r="E125" s="685" t="inlineStr">
         <is>
-          <t>- Đóng popup, ở lại màn chi tiết
+          <t>2. 
+- Đóng popup, ở lại màn chi tiết
 - Trạng thái gói giữ nguyên "Nháp", không lưu thay đổi
 - Button Phát hành vẫn hiển thị</t>
         </is>
@@ -8001,7 +8014,7 @@
       </c>
       <c r="E126" s="685" t="inlineStr">
         <is>
-          <t>Cả 5 trường hợp đều đóng popup, gói giữ trạng thái Nháp</t>
+          <t>2. Cả 5 trường hợp đều đóng popup, gói giữ trạng thái Nháp</t>
         </is>
       </c>
       <c r="F126" s="683" t="n"/>
@@ -8044,7 +8057,7 @@
       </c>
       <c r="E127" s="685" t="inlineStr">
         <is>
-          <t>Đóng popup, gói giữ trạng thái Nháp</t>
+          <t>2. Đóng popup, gói giữ trạng thái Nháp</t>
         </is>
       </c>
       <c r="F127" s="683" t="n"/>
@@ -8087,7 +8100,7 @@
       </c>
       <c r="E128" s="685" t="inlineStr">
         <is>
-          <t>Đóng popup, gói giữ trạng thái Nháp</t>
+          <t>2. Đóng popup, gói giữ trạng thái Nháp</t>
         </is>
       </c>
       <c r="F128" s="683" t="n"/>
@@ -8127,7 +8140,7 @@
       </c>
       <c r="E129" s="685" t="inlineStr">
         <is>
-          <t>Popup hiển thị lại đúng nội dung theo trường hợp của gói</t>
+          <t>3. Popup hiển thị lại đúng nội dung theo trường hợp của gói</t>
         </is>
       </c>
       <c r="F129" s="683" t="n"/>
@@ -8166,7 +8179,7 @@
       <c r="L130" s="683" t="n"/>
       <c r="M130" s="683" t="n"/>
     </row>
-    <row r="131" ht="64" customHeight="1" s="668">
+    <row r="131" ht="80" customHeight="1" s="668">
       <c r="A131" s="684">
         <f>$C$4&amp;"-"&amp;TEXT(COUNTA($D$12:D131),"00")</f>
         <v/>
@@ -8189,7 +8202,8 @@
       </c>
       <c r="E131" s="685" t="inlineStr">
         <is>
-          <t>- status = trạng thái mới đúng rule
+          <t>2. 
+- status = trạng thái mới đúng rule
 - updated_by = Admin phát hành
 - updated_at = thời điểm xác nhận
 - Các trường khác không đổi</t>
@@ -8231,7 +8245,7 @@
       </c>
       <c r="E132" s="685" t="inlineStr">
         <is>
-          <t>Cột Trạng thái, Thời gian cập nhật, Người cập nhật của gói hiển thị giá trị mới</t>
+          <t>2. Cột Trạng thái, Thời gian cập nhật, Người cập nhật của gói hiển thị giá trị mới</t>
         </is>
       </c>
       <c r="F132" s="683" t="n"/>
@@ -8270,7 +8284,7 @@
       </c>
       <c r="E133" s="685" t="inlineStr">
         <is>
-          <t>Ghi log: người thao tác, thời gian, IP, trạng thái cũ (Nháp) → mới</t>
+          <t>2. Ghi log: người thao tác, thời gian, IP, trạng thái cũ (Nháp) → mới</t>
         </is>
       </c>
       <c r="F133" s="683" t="n"/>
@@ -8313,7 +8327,7 @@
       </c>
       <c r="E134" s="685" t="inlineStr">
         <is>
-          <t>Chỉ gửi 1 yêu cầu, gói chuyển trạng thái 1 lần, chỉ 1 toast thành công</t>
+          <t>2. Chỉ gửi 1 yêu cầu, gói chuyển trạng thái 1 lần, chỉ 1 toast thành công</t>
         </is>
       </c>
       <c r="F134" s="683" t="n"/>
@@ -8356,7 +8370,7 @@
       </c>
       <c r="E135" s="685" t="inlineStr">
         <is>
-          <t>Hiển thị toast "Phát hành gói cước thành công", tự ẩn sau vài giây</t>
+          <t>2. Hiển thị toast "Phát hành gói cước thành công", tự ẩn sau vài giây</t>
         </is>
       </c>
       <c r="F135" s="683" t="n"/>
@@ -8400,8 +8414,8 @@
       </c>
       <c r="E136" s="685" t="inlineStr">
         <is>
-          <t>- Không có button Phát hành
-- API trả lỗi, trạng thái gói không đổi</t>
+          <t>1. Không hiển thị button Phát hành
+2. API trả lỗi, trạng thái gói không đổi</t>
         </is>
       </c>
       <c r="F136" s="683" t="n"/>
@@ -8440,7 +8454,7 @@
       </c>
       <c r="E137" s="685" t="inlineStr">
         <is>
-          <t>Không cho phép phát hành, hiển thị thông báo lỗi; gói giữ Đã xoá</t>
+          <t>1. Không cho phép phát hành, hiển thị thông báo lỗi; gói giữ Đã xoá</t>
         </is>
       </c>
       <c r="F137" s="683" t="n"/>
@@ -8484,8 +8498,8 @@
       </c>
       <c r="E138" s="685" t="inlineStr">
         <is>
-          <t>- A phát hành thành công
-- B nhận thông báo lỗi, không phát sinh chuyển trạng thái lần 2</t>
+          <t>1. A phát hành thành công, toast "Phát hành gói cước thành công"
+2. B nhận thông báo lỗi, không phát sinh chuyển trạng thái lần 2</t>
         </is>
       </c>
       <c r="F138" s="683" t="n"/>
@@ -8524,7 +8538,7 @@
       </c>
       <c r="E139" s="685" t="inlineStr">
         <is>
-          <t>Hệ thống xử lý theo dữ liệu mới nhất trong DB (gói chuyển Ngừng kinh doanh) hoặc yêu cầu A tải lại trang</t>
+          <t>1. Hệ thống xử lý theo dữ liệu mới nhất trong DB (gói chuyển Ngừng kinh doanh) hoặc yêu cầu A tải lại trang</t>
         </is>
       </c>
       <c r="F139" s="683" t="n"/>
@@ -8567,7 +8581,7 @@
       </c>
       <c r="E140" s="685" t="inlineStr">
         <is>
-          <t>Chặn phát hành, báo gói chưa cấu hình đủ tham số</t>
+          <t>1. Chặn phát hành, báo gói chưa cấu hình đủ tham số</t>
         </is>
       </c>
       <c r="F140" s="683" t="n"/>
@@ -8611,7 +8625,8 @@
       </c>
       <c r="E141" s="685" t="inlineStr">
         <is>
-          <t>- Hiển thị toast "Thất bại. Vui lòng kiểm tra lại kết nối."
+          <t>3. 
+- Hiển thị toast "Thất bại. Vui lòng kiểm tra lại kết nối."
 - Gói giữ Nháp, cho phép click lại</t>
         </is>
       </c>
@@ -8652,7 +8667,7 @@
       </c>
       <c r="E142" s="685" t="inlineStr">
         <is>
-          <t>Phát hành thành công, toast "Phát hành gói cước thành công"</t>
+          <t>2. Phát hành thành công, toast "Phát hành gói cước thành công"</t>
         </is>
       </c>
       <c r="F142" s="683" t="n"/>
@@ -8695,7 +8710,8 @@
       </c>
       <c r="E143" s="685" t="inlineStr">
         <is>
-          <t>- Hiển thị toast "Hệ thống bận. Vui lòng thử lại sau." kèm mã lỗi
+          <t>1. 
+- Hiển thị toast "Hệ thống bận. Vui lòng thử lại sau." kèm mã lỗi
 - Gói giữ Nháp, cho phép click lại</t>
         </is>
       </c>
@@ -8739,7 +8755,7 @@
       </c>
       <c r="E144" s="685" t="inlineStr">
         <is>
-          <t>Không hiển thị button Phát hành / gọi API bị từ chối</t>
+          <t>1. Không hiển thị button Phát hành / gọi API bị từ chối</t>
         </is>
       </c>
       <c r="F144" s="683" t="n"/>
@@ -8783,7 +8799,7 @@
       </c>
       <c r="E145" s="685" t="inlineStr">
         <is>
-          <t>Không cho sửa Mã gói, Loại gói, Tham số</t>
+          <t>2. Không cho sửa Mã gói, Loại gói, Tham số</t>
         </is>
       </c>
       <c r="F145" s="683" t="n"/>
@@ -8823,7 +8839,7 @@
       </c>
       <c r="E146" s="685" t="inlineStr">
         <is>
-          <t>Không cho sửa Mã gói, Chu kỳ, Loại hình</t>
+          <t>2. Không cho sửa Mã gói, Chu kỳ, Loại hình</t>
         </is>
       </c>
       <c r="F146" s="683" t="n"/>

</xml_diff>